<commit_message>
job aps cover letters and comp mod guest lecture
</commit_message>
<xml_diff>
--- a/data/complementarity/complimentarity_setup_mar2.xlsx
+++ b/data/complementarity/complimentarity_setup_mar2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timet\Documents\projectCSUN\csunThesisRepo\data\complementarity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4EDB5E-E546-4F3B-89E7-B4E2B64BCEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30AD3FA0-BC2F-4163-804E-832769C360E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55E80E2A-D0E6-46F0-8B77-35CBC3976946}"/>
+    <workbookView xWindow="795" yWindow="2025" windowWidth="25500" windowHeight="12675" xr2:uid="{55E80E2A-D0E6-46F0-8B77-35CBC3976946}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="63">
   <si>
     <t>clone</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>BLOCK 2</t>
+  </si>
+  <si>
+    <t>BLOCK 3</t>
   </si>
 </sst>
 </file>
@@ -234,7 +237,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -246,21 +249,6 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="2" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -279,7 +267,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -307,6 +295,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -370,9 +364,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -387,16 +378,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -736,14 +730,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A89CF7-398C-4C16-BC5E-A2E563F1A358}">
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="10" max="10" width="9.625" customWidth="1"/>
     <col min="11" max="12" width="13.125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.25" bestFit="1" customWidth="1"/>
@@ -830,23 +824,23 @@
         <f>400/F3</f>
         <v>2.1176470588235294</v>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="7">
         <f>I3/5</f>
         <v>0.42352941176470588</v>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="7">
         <f>20-(I3+G3+H3)</f>
         <v>16.046638655462186</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="7">
         <f>K3+H3</f>
         <v>17.83235294117647</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="6">
         <f>20-(H3+(SUM(J3:J7))+G3)</f>
         <v>15.776388664990193</v>
       </c>
-      <c r="N3" s="8">
+      <c r="N3" s="5">
         <f>M3-H3</f>
         <v>13.990674379275907</v>
       </c>
@@ -883,15 +877,15 @@
         <f t="shared" ref="I4:I7" si="1">400/F4</f>
         <v>3.3962264150943393</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="7">
         <f t="shared" ref="J4:J7" si="2">I4/5</f>
         <v>0.67924528301886788</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="7">
         <f>20-(I4+G4+H4)</f>
         <v>14.768059299191375</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="7">
         <f t="shared" ref="L4:L7" si="3">K4+H4</f>
         <v>16.55377358490566</v>
       </c>
@@ -930,15 +924,15 @@
         <f>400/F5</f>
         <v>2.2360248447204971</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="7">
         <f t="shared" si="2"/>
         <v>0.44720496894409945</v>
       </c>
-      <c r="K5" s="10">
+      <c r="K5" s="7">
         <f>20-(I5+G5+H5)</f>
         <v>15.928260869565218</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5" s="7">
         <f t="shared" si="3"/>
         <v>17.713975155279503</v>
       </c>
@@ -977,15 +971,15 @@
         <f t="shared" si="1"/>
         <v>2.1556886227544911</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="7">
         <f t="shared" si="2"/>
         <v>0.43113772455089822</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="7">
         <f>20-(I6+G6+H6)</f>
         <v>16.008597091531222</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="7">
         <f t="shared" si="3"/>
         <v>17.794311377245506</v>
       </c>
@@ -1024,15 +1018,15 @@
         <f t="shared" si="1"/>
         <v>2.0338983050847457</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="7">
         <f t="shared" si="2"/>
         <v>0.40677966101694912</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="8">
         <f>20-(I7+G7+H7)</f>
         <v>16.130387409200971</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L7" s="7">
         <f t="shared" si="3"/>
         <v>17.916101694915255</v>
       </c>
@@ -1040,20 +1034,15 @@
       <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="A8" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="29"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
     </row>
@@ -1102,46 +1091,46 @@
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
-        <v>16</v>
-      </c>
-      <c r="B10" s="12">
+      <c r="A10" s="9">
+        <v>16</v>
+      </c>
+      <c r="B10" s="9">
         <v>26</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="9">
         <v>18</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="9">
         <v>26</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="10">
         <f>AVERAGE(B10:D10)</f>
         <v>23.333333333333332</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="10">
         <f>E10*10</f>
         <v>233.33333333333331</v>
       </c>
-      <c r="G10" s="12">
-        <v>0</v>
-      </c>
-      <c r="H10" s="12">
+      <c r="G10" s="9">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9">
         <f>800/5757</f>
         <v>0.13896126454750737</v>
       </c>
-      <c r="I10" s="14">
+      <c r="I10" s="11">
         <f>400/F10</f>
         <v>1.7142857142857144</v>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="11">
         <f>I10/5</f>
         <v>0.34285714285714286</v>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="18">
         <f>20 - (H10+I10)</f>
         <v>18.146753021166777</v>
       </c>
-      <c r="L10" s="21">
+      <c r="L10" s="18">
         <f>(20-I10)</f>
         <v>18.285714285714285</v>
       </c>
@@ -1161,47 +1150,47 @@
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
+      <c r="A11" s="9">
         <v>3</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="9">
         <v>46</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="9">
         <v>45</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="9">
         <v>34</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="10">
         <f>AVERAGE(B11:D11)</f>
         <v>41.666666666666664</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="10">
         <f t="shared" ref="F11:F14" si="4">E11*10</f>
         <v>416.66666666666663</v>
       </c>
-      <c r="G11" s="12">
-        <v>0</v>
-      </c>
-      <c r="H11" s="12">
+      <c r="G11" s="9">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
         <f t="shared" ref="H11:H14" si="5">800/5757</f>
         <v>0.13896126454750737</v>
       </c>
-      <c r="I11" s="14">
+      <c r="I11" s="11">
         <f t="shared" ref="I11:I14" si="6">400/F11</f>
         <v>0.96000000000000008</v>
       </c>
-      <c r="J11" s="14">
-        <f t="shared" ref="J11:J14" si="7">I11/5</f>
+      <c r="J11" s="11">
+        <f>I11/5</f>
         <v>0.192</v>
       </c>
-      <c r="K11" s="21">
-        <f t="shared" ref="K11:K14" si="8">20 - (H11+I11)</f>
+      <c r="K11" s="18">
+        <f t="shared" ref="K11:K14" si="7">20 - (H11+I11)</f>
         <v>18.901038735452492</v>
       </c>
-      <c r="L11" s="21">
-        <f t="shared" ref="L11:L14" si="9">(20-I11)</f>
+      <c r="L11" s="18">
+        <f t="shared" ref="L11:L14" si="8">(20-I11)</f>
         <v>19.04</v>
       </c>
       <c r="P11">
@@ -1217,159 +1206,159 @@
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
+      <c r="A12" s="9">
         <v>2</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="9">
         <v>31</v>
       </c>
-      <c r="C12" s="12">
-        <v>28</v>
-      </c>
-      <c r="D12" s="12">
+      <c r="C12" s="9">
+        <v>28</v>
+      </c>
+      <c r="D12" s="9">
         <v>24</v>
       </c>
-      <c r="E12" s="13">
-        <f t="shared" ref="E12:E14" si="10">AVERAGE(B12:D12)</f>
+      <c r="E12" s="10">
+        <f t="shared" ref="E12:E14" si="9">AVERAGE(B12:D12)</f>
         <v>27.666666666666668</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="10">
         <f t="shared" si="4"/>
         <v>276.66666666666669</v>
       </c>
-      <c r="G12" s="12">
-        <v>0</v>
-      </c>
-      <c r="H12" s="12">
+      <c r="G12" s="9">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
         <f t="shared" si="5"/>
         <v>0.13896126454750737</v>
       </c>
-      <c r="I12" s="14">
+      <c r="I12" s="11">
         <f t="shared" si="6"/>
         <v>1.4457831325301205</v>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="11">
         <f>I12/5</f>
         <v>0.28915662650602408</v>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="18">
+        <f t="shared" si="7"/>
+        <v>18.415255602922372</v>
+      </c>
+      <c r="L12" s="18">
         <f t="shared" si="8"/>
-        <v>18.415255602922372</v>
-      </c>
-      <c r="L12" s="21">
-        <f t="shared" si="9"/>
         <v>18.554216867469879</v>
       </c>
       <c r="P12">
         <v>79</v>
       </c>
       <c r="Q12">
-        <f t="shared" ref="Q12:Q13" si="11">P12*6.8</f>
+        <f t="shared" ref="Q12:Q13" si="10">P12*6.8</f>
         <v>537.19999999999993</v>
       </c>
       <c r="R12">
-        <f t="shared" ref="R12:R13" si="12">Q12*10</f>
+        <f t="shared" ref="R12:R13" si="11">Q12*10</f>
         <v>5371.9999999999991</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
+      <c r="A13" s="9">
         <v>14</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="9">
         <v>32</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="9">
         <v>25</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="9">
         <v>21</v>
       </c>
-      <c r="E13" s="13">
-        <f t="shared" si="10"/>
+      <c r="E13" s="10">
+        <f t="shared" si="9"/>
         <v>26</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="10">
         <f t="shared" si="4"/>
         <v>260</v>
       </c>
-      <c r="G13" s="12">
-        <v>0</v>
-      </c>
-      <c r="H13" s="12">
+      <c r="G13" s="9">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9">
         <f t="shared" si="5"/>
         <v>0.13896126454750737</v>
       </c>
-      <c r="I13" s="14">
+      <c r="I13" s="11">
         <f t="shared" si="6"/>
         <v>1.5384615384615385</v>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="11">
+        <f t="shared" ref="J11:J14" si="12">I13/5</f>
+        <v>0.30769230769230771</v>
+      </c>
+      <c r="K13" s="18">
         <f t="shared" si="7"/>
-        <v>0.30769230769230771</v>
-      </c>
-      <c r="K13" s="21">
+        <v>18.322577196990956</v>
+      </c>
+      <c r="L13" s="18">
         <f t="shared" si="8"/>
-        <v>18.322577196990956</v>
-      </c>
-      <c r="L13" s="21">
-        <f t="shared" si="9"/>
         <v>18.46153846153846</v>
       </c>
       <c r="P13">
         <v>88</v>
       </c>
       <c r="Q13">
+        <f t="shared" si="10"/>
+        <v>598.4</v>
+      </c>
+      <c r="R13">
         <f t="shared" si="11"/>
-        <v>598.4</v>
-      </c>
-      <c r="R13">
-        <f t="shared" si="12"/>
         <v>5984</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="9">
         <v>5</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="9">
         <v>25</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="9">
         <v>24</v>
       </c>
-      <c r="D14" s="12">
-        <v>28</v>
-      </c>
-      <c r="E14" s="13">
-        <f t="shared" si="10"/>
+      <c r="D14" s="9">
+        <v>28</v>
+      </c>
+      <c r="E14" s="10">
+        <f t="shared" si="9"/>
         <v>25.666666666666668</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <f t="shared" si="4"/>
         <v>256.66666666666669</v>
       </c>
-      <c r="G14" s="12">
-        <v>0</v>
-      </c>
-      <c r="H14" s="12">
+      <c r="G14" s="9">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9">
         <f t="shared" si="5"/>
         <v>0.13896126454750737</v>
       </c>
-      <c r="I14" s="14">
+      <c r="I14" s="11">
         <f t="shared" si="6"/>
         <v>1.5584415584415583</v>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="11">
+        <f t="shared" si="12"/>
+        <v>0.31168831168831168</v>
+      </c>
+      <c r="K14" s="18">
         <f t="shared" si="7"/>
-        <v>0.31168831168831168</v>
-      </c>
-      <c r="K14" s="21">
+        <v>18.302597177010934</v>
+      </c>
+      <c r="L14" s="18">
         <f t="shared" si="8"/>
-        <v>18.302597177010934</v>
-      </c>
-      <c r="L14" s="21">
-        <f t="shared" si="9"/>
         <v>18.441558441558442</v>
       </c>
       <c r="R14">
@@ -1381,20 +1370,15 @@
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" s="26" t="s">
+      <c r="A15" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1441,46 +1425,46 @@
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="12">
         <v>7</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="12">
         <v>129</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="12">
         <v>116</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="12">
         <v>79</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="12">
         <f>AVERAGE(B17:D17)</f>
         <v>108</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="13">
         <f>E17/0.3</f>
         <v>360</v>
       </c>
-      <c r="G17" s="15">
-        <v>0</v>
-      </c>
-      <c r="H17" s="15">
+      <c r="G17" s="12">
+        <v>0</v>
+      </c>
+      <c r="H17" s="12">
         <f>800/3128</f>
         <v>0.25575447570332482</v>
       </c>
-      <c r="I17" s="17">
+      <c r="I17" s="14">
         <f>400/F17</f>
         <v>1.1111111111111112</v>
       </c>
-      <c r="J17" s="17">
+      <c r="J17" s="14">
         <f>I17/5</f>
         <v>0.22222222222222224</v>
       </c>
-      <c r="K17" s="22">
+      <c r="K17" s="19">
         <f>20 - (H17+I17)</f>
         <v>18.633134413185566</v>
       </c>
-      <c r="L17" s="22">
+      <c r="L17" s="19">
         <f>(20-I17)</f>
         <v>18.888888888888889</v>
       </c>
@@ -1500,46 +1484,46 @@
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="12">
         <v>8</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="12">
         <v>70</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="12">
         <v>78</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="12">
         <v>91</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="12">
         <f t="shared" ref="E18:E21" si="13">AVERAGE(B18:D18)</f>
         <v>79.666666666666671</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="13">
         <f>E18/0.3</f>
         <v>265.5555555555556</v>
       </c>
-      <c r="G18" s="15">
-        <v>0</v>
-      </c>
-      <c r="H18" s="15">
+      <c r="G18" s="12">
+        <v>0</v>
+      </c>
+      <c r="H18" s="12">
         <f t="shared" ref="H18:H21" si="14">800/3128</f>
         <v>0.25575447570332482</v>
       </c>
-      <c r="I18" s="17">
+      <c r="I18" s="14">
         <f t="shared" ref="I18:I21" si="15">400/F18</f>
         <v>1.5062761506276148</v>
       </c>
-      <c r="J18" s="17">
+      <c r="J18" s="14">
         <f t="shared" ref="J18:J21" si="16">I18/5</f>
         <v>0.30125523012552297</v>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="19">
         <f t="shared" ref="K18:K21" si="17">20 - (H18+I18)</f>
         <v>18.23796937366906</v>
       </c>
-      <c r="L18" s="22">
+      <c r="L18" s="19">
         <f t="shared" ref="L18:L21" si="18">(20-I18)</f>
         <v>18.493723849372387</v>
       </c>
@@ -1556,46 +1540,46 @@
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="12">
         <v>9</v>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="12">
         <v>71</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="12">
         <v>105</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="12">
         <v>70</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="12">
         <f>AVERAGE(B19:D19)</f>
         <v>82</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="13">
         <f>E19/0.3</f>
         <v>273.33333333333337</v>
       </c>
-      <c r="G19" s="15">
-        <v>0</v>
-      </c>
-      <c r="H19" s="15">
+      <c r="G19" s="12">
+        <v>0</v>
+      </c>
+      <c r="H19" s="12">
         <f t="shared" si="14"/>
         <v>0.25575447570332482</v>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="14">
         <f t="shared" si="15"/>
         <v>1.4634146341463412</v>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="14">
         <f t="shared" si="16"/>
         <v>0.29268292682926822</v>
       </c>
-      <c r="K19" s="22">
+      <c r="K19" s="19">
         <f t="shared" si="17"/>
         <v>18.280830890150334</v>
       </c>
-      <c r="L19" s="22">
+      <c r="L19" s="19">
         <f t="shared" si="18"/>
         <v>18.536585365853657</v>
       </c>
@@ -1612,46 +1596,46 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="12">
         <v>10</v>
       </c>
-      <c r="B20" s="23">
+      <c r="B20" s="20">
         <v>61</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="12">
         <v>102</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="12">
         <v>58</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="12">
         <f t="shared" si="13"/>
         <v>73.666666666666671</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="13">
         <f>E20/0.3</f>
         <v>245.55555555555557</v>
       </c>
-      <c r="G20" s="15">
-        <v>0</v>
-      </c>
-      <c r="H20" s="15">
+      <c r="G20" s="12">
+        <v>0</v>
+      </c>
+      <c r="H20" s="12">
         <f t="shared" si="14"/>
         <v>0.25575447570332482</v>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="14">
         <f t="shared" si="15"/>
         <v>1.6289592760180995</v>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="14">
         <f t="shared" si="16"/>
         <v>0.32579185520361992</v>
       </c>
-      <c r="K20" s="22">
+      <c r="K20" s="19">
         <f t="shared" si="17"/>
         <v>18.115286248278576</v>
       </c>
-      <c r="L20" s="22">
+      <c r="L20" s="19">
         <f t="shared" si="18"/>
         <v>18.371040723981899</v>
       </c>
@@ -1668,46 +1652,46 @@
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="12">
         <v>15</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="12">
         <v>62</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="12">
         <v>86</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="12">
         <v>60</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="12">
         <f t="shared" si="13"/>
         <v>69.333333333333329</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="13">
         <f>E21/0.3</f>
         <v>231.11111111111111</v>
       </c>
-      <c r="G21" s="15">
-        <v>0</v>
-      </c>
-      <c r="H21" s="15">
+      <c r="G21" s="12">
+        <v>0</v>
+      </c>
+      <c r="H21" s="12">
         <f t="shared" si="14"/>
         <v>0.25575447570332482</v>
       </c>
-      <c r="I21" s="17">
+      <c r="I21" s="14">
         <f t="shared" si="15"/>
         <v>1.7307692307692308</v>
       </c>
-      <c r="J21" s="17">
+      <c r="J21" s="14">
         <f t="shared" si="16"/>
         <v>0.34615384615384615</v>
       </c>
-      <c r="K21" s="22">
+      <c r="K21" s="19">
         <f t="shared" si="17"/>
         <v>18.013476293527443</v>
       </c>
-      <c r="L21" s="22">
+      <c r="L21" s="19">
         <f t="shared" si="18"/>
         <v>18.26923076923077</v>
       </c>
@@ -1720,30 +1704,291 @@
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="5">
+      <c r="F24" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" t="s">
+        <v>6</v>
+      </c>
+      <c r="H24" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" t="s">
+        <v>8</v>
+      </c>
+      <c r="J24" t="s">
+        <v>11</v>
+      </c>
+      <c r="K24" t="s">
+        <v>9</v>
+      </c>
+      <c r="L24" t="s">
+        <v>10</v>
+      </c>
+      <c r="M24" t="s">
+        <v>12</v>
+      </c>
+      <c r="N24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25" s="25">
+        <v>1</v>
+      </c>
+      <c r="B25" s="25">
+        <v>44</v>
+      </c>
+      <c r="C25" s="25">
+        <v>36</v>
+      </c>
+      <c r="D25" s="25">
+        <v>71</v>
+      </c>
+      <c r="E25" s="25">
+        <f>AVERAGE(B25:D25)</f>
+        <v>50.333333333333336</v>
+      </c>
+      <c r="F25" s="26">
+        <f>E25/0.3</f>
+        <v>167.7777777777778</v>
+      </c>
+      <c r="G25" s="25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="25">
+        <f>800/4352</f>
+        <v>0.18382352941176472</v>
+      </c>
+      <c r="I25" s="27">
+        <f>400/F25</f>
+        <v>2.3841059602649004</v>
+      </c>
+      <c r="J25" s="27">
+        <f>I25/5</f>
+        <v>0.47682119205298007</v>
+      </c>
+      <c r="K25" s="28">
+        <f>20 - (H25+I25)</f>
+        <v>17.432070510323335</v>
+      </c>
+      <c r="L25" s="28">
+        <f>(20-I25)</f>
+        <v>17.6158940397351</v>
+      </c>
+      <c r="M25" s="1">
+        <f>20-(SUM(J25:J29)+H25)</f>
+        <v>17.734336368635368</v>
+      </c>
+      <c r="N25" s="1">
+        <f>20-SUM(J25:J29)</f>
+        <v>17.918159898047129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26" s="25">
+        <v>11</v>
+      </c>
+      <c r="B26" s="25">
+        <v>73</v>
+      </c>
+      <c r="C26" s="25">
+        <v>62</v>
+      </c>
+      <c r="D26" s="25">
+        <v>82</v>
+      </c>
+      <c r="E26" s="25">
+        <f t="shared" ref="E26:E29" si="21">AVERAGE(B26:D26)</f>
+        <v>72.333333333333329</v>
+      </c>
+      <c r="F26" s="26">
+        <f>E26/0.3</f>
+        <v>241.11111111111111</v>
+      </c>
+      <c r="G26" s="25">
+        <v>0</v>
+      </c>
+      <c r="H26" s="25">
+        <f t="shared" ref="H26:H29" si="22">800/4352</f>
+        <v>0.18382352941176472</v>
+      </c>
+      <c r="I26" s="27">
+        <f t="shared" ref="I26:I29" si="23">400/F26</f>
+        <v>1.6589861751152073</v>
+      </c>
+      <c r="J26" s="27">
+        <f t="shared" ref="J26:J29" si="24">I26/5</f>
+        <v>0.33179723502304148</v>
+      </c>
+      <c r="K26" s="28">
+        <f t="shared" ref="K26:K29" si="25">20 - (H26+I26)</f>
+        <v>18.157190295473029</v>
+      </c>
+      <c r="L26" s="28">
+        <f t="shared" ref="L26:L29" si="26">(20-I26)</f>
+        <v>18.341013824884794</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="25">
+        <v>6</v>
+      </c>
+      <c r="B27" s="25">
+        <v>60</v>
+      </c>
+      <c r="C27" s="25">
+        <v>50</v>
+      </c>
+      <c r="D27" s="25">
+        <v>64</v>
+      </c>
+      <c r="E27" s="25">
+        <f>AVERAGE(B27:D27)</f>
+        <v>58</v>
+      </c>
+      <c r="F27" s="26">
+        <f>E27/0.3</f>
+        <v>193.33333333333334</v>
+      </c>
+      <c r="G27" s="25">
+        <v>0</v>
+      </c>
+      <c r="H27" s="25">
+        <f t="shared" si="22"/>
+        <v>0.18382352941176472</v>
+      </c>
+      <c r="I27" s="27">
+        <f t="shared" si="23"/>
+        <v>2.068965517241379</v>
+      </c>
+      <c r="J27" s="27">
+        <f t="shared" si="24"/>
+        <v>0.4137931034482758</v>
+      </c>
+      <c r="K27" s="28">
+        <f t="shared" si="25"/>
+        <v>17.747210953346858</v>
+      </c>
+      <c r="L27" s="28">
+        <f t="shared" si="26"/>
+        <v>17.931034482758619</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A28" s="25">
+        <v>4</v>
+      </c>
+      <c r="B28" s="29">
+        <v>80</v>
+      </c>
+      <c r="C28" s="25">
+        <v>94</v>
+      </c>
+      <c r="D28" s="25">
+        <v>76</v>
+      </c>
+      <c r="E28" s="25">
+        <f t="shared" ref="E28:E29" si="27">AVERAGE(B28:D28)</f>
+        <v>83.333333333333329</v>
+      </c>
+      <c r="F28" s="26">
+        <f>E28/0.3</f>
+        <v>277.77777777777777</v>
+      </c>
+      <c r="G28" s="25">
+        <v>0</v>
+      </c>
+      <c r="H28" s="25">
+        <f t="shared" si="22"/>
+        <v>0.18382352941176472</v>
+      </c>
+      <c r="I28" s="27">
+        <f t="shared" si="23"/>
+        <v>1.44</v>
+      </c>
+      <c r="J28" s="27">
+        <f t="shared" si="24"/>
+        <v>0.28799999999999998</v>
+      </c>
+      <c r="K28" s="28">
+        <f t="shared" si="25"/>
+        <v>18.376176470588234</v>
+      </c>
+      <c r="L28" s="28">
+        <f t="shared" si="26"/>
+        <v>18.559999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A29" s="25">
+        <v>17</v>
+      </c>
+      <c r="B29" s="25">
+        <v>24</v>
+      </c>
+      <c r="C29" s="25">
+        <v>47</v>
+      </c>
+      <c r="D29" s="25">
+        <v>55</v>
+      </c>
+      <c r="E29" s="25">
+        <f t="shared" si="27"/>
         <v>42</v>
       </c>
-      <c r="C23" s="5">
-        <v>47</v>
-      </c>
-      <c r="D23" s="5">
-        <v>54</v>
-      </c>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6">
-        <f>E23/0.3</f>
-        <v>0</v>
-      </c>
-      <c r="G23" s="5">
-        <v>0.05</v>
-      </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="7" t="e">
-        <f>800/F23</f>
-        <v>#DIV/0!</v>
+      <c r="F29" s="26">
+        <f>E29/0.3</f>
+        <v>140</v>
+      </c>
+      <c r="G29" s="25">
+        <v>0</v>
+      </c>
+      <c r="H29" s="25">
+        <f t="shared" si="22"/>
+        <v>0.18382352941176472</v>
+      </c>
+      <c r="I29" s="27">
+        <f t="shared" si="23"/>
+        <v>2.8571428571428572</v>
+      </c>
+      <c r="J29" s="27">
+        <f t="shared" si="24"/>
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="K29" s="28">
+        <f t="shared" si="25"/>
+        <v>16.959033613445378</v>
+      </c>
+      <c r="L29" s="28">
+        <f t="shared" si="26"/>
+        <v>17.142857142857142</v>
       </c>
     </row>
   </sheetData>
@@ -1765,7 +2010,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="21" t="s">
         <v>55</v>
       </c>
       <c r="B1" t="s">
@@ -1774,12 +2019,12 @@
       <c r="C1" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="21" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="24">
+      <c r="A2" s="21">
         <v>7</v>
       </c>
       <c r="B2">
@@ -1788,13 +2033,13 @@
       <c r="C2" s="1">
         <v>1.1111111111111112</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="22">
         <f>C2/2*100</f>
         <v>55.555555555555557</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="24">
+      <c r="A3" s="21">
         <v>8</v>
       </c>
       <c r="B3">
@@ -1803,13 +2048,13 @@
       <c r="C3" s="1">
         <v>1.5062761506276148</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="22">
         <f t="shared" ref="D3:D6" si="0">C3/2*100</f>
         <v>75.313807531380732</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="24">
+      <c r="A4" s="21">
         <v>9</v>
       </c>
       <c r="B4">
@@ -1818,13 +2063,13 @@
       <c r="C4" s="1">
         <v>1.4634146341463412</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="22">
         <f t="shared" si="0"/>
         <v>73.17073170731706</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="24">
+      <c r="A5" s="21">
         <v>10</v>
       </c>
       <c r="B5">
@@ -1833,13 +2078,13 @@
       <c r="C5" s="1">
         <v>1.6289592760180995</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="22">
         <f t="shared" si="0"/>
         <v>81.447963800904972</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="24">
+      <c r="A6" s="21">
         <v>15</v>
       </c>
       <c r="B6">
@@ -1848,7 +2093,7 @@
       <c r="C6" s="1">
         <v>1.7307692307692308</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="22">
         <f t="shared" si="0"/>
         <v>86.538461538461547</v>
       </c>
@@ -1873,7 +2118,7 @@
       <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E1" t="s">
@@ -1882,19 +2127,19 @@
       <c r="F1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="15" t="s">
         <v>26</v>
       </c>
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -3183,7 +3428,7 @@
       <c r="E48">
         <v>5</v>
       </c>
-      <c r="F48" s="19" t="s">
+      <c r="F48" s="16" t="s">
         <v>31</v>
       </c>
       <c r="G48" t="s">
@@ -3212,7 +3457,7 @@
       <c r="E49">
         <v>6</v>
       </c>
-      <c r="F49" s="19" t="s">
+      <c r="F49" s="16" t="s">
         <v>32</v>
       </c>
       <c r="G49" t="s">
@@ -4016,7 +4261,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4048,10 +4293,10 @@
       <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="20"/>
+      <c r="I1" s="17"/>
     </row>
     <row r="2" spans="1:9" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -4066,16 +4311,16 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="20">
+      <c r="H2" s="17">
         <v>107</v>
       </c>
-      <c r="I2" s="20"/>
+      <c r="I2" s="17"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">

</xml_diff>